<commit_message>
updated files ira modeling
</commit_message>
<xml_diff>
--- a/InputData/trans/BPHEVSP/BAU PHEV Subsidy Perc.xlsx
+++ b/InputData/trans/BPHEVSP/BAU PHEV Subsidy Perc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-arizona\InputData\trans\BPHEVSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\PA\trans\BPHEVSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6867B4ED-8421-4086-B2EB-E5C9C793786A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC4B63B7-05D8-49CA-B4C7-1B9A0C4B9EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31080" yWindow="2280" windowWidth="23085" windowHeight="13305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="360" windowWidth="14400" windowHeight="7350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="193">
   <si>
     <t>Sources:</t>
   </si>
@@ -355,6 +355,267 @@
   <si>
     <t>Subsidy goes up to 2000 based on battery &amp; price</t>
   </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>Alabama</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>Alaska</t>
+  </si>
+  <si>
+    <t>AK</t>
+  </si>
+  <si>
+    <t>Arizona</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>Arkansas</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Connecticut</t>
+  </si>
+  <si>
+    <t>Delaware</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>GA</t>
+  </si>
+  <si>
+    <t>Hawaii</t>
+  </si>
+  <si>
+    <t>HI</t>
+  </si>
+  <si>
+    <t>Idaho</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>IL</t>
+  </si>
+  <si>
+    <t>Indiana</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>Iowa</t>
+  </si>
+  <si>
+    <t>IA</t>
+  </si>
+  <si>
+    <t>Kansas</t>
+  </si>
+  <si>
+    <t>KS</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
+  </si>
+  <si>
+    <t>KY</t>
+  </si>
+  <si>
+    <t>Louisiana</t>
+  </si>
+  <si>
+    <t>Maine</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>Michigan</t>
+  </si>
+  <si>
+    <t>MI</t>
+  </si>
+  <si>
+    <t>Minnesota</t>
+  </si>
+  <si>
+    <t>MN</t>
+  </si>
+  <si>
+    <t>Mississippi</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>Missouri</t>
+  </si>
+  <si>
+    <t>MO</t>
+  </si>
+  <si>
+    <t>Montana</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>Nebraska</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>NV</t>
+  </si>
+  <si>
+    <t>New Hampshire</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>New Jersey</t>
+  </si>
+  <si>
+    <t>New Mexico</t>
+  </si>
+  <si>
+    <t>NM</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>North Carolina</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t>North Dakota</t>
+  </si>
+  <si>
+    <t>ND</t>
+  </si>
+  <si>
+    <t>Ohio</t>
+  </si>
+  <si>
+    <t>OH</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Oregon</t>
+  </si>
+  <si>
+    <t>Pennsylvania</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
+    <t>RI</t>
+  </si>
+  <si>
+    <t>South Carolina</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>South Dakota</t>
+  </si>
+  <si>
+    <t>SD</t>
+  </si>
+  <si>
+    <t>Tennessee</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Utah</t>
+  </si>
+  <si>
+    <t>UT</t>
+  </si>
+  <si>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>VA</t>
+  </si>
+  <si>
+    <t>Washington</t>
+  </si>
+  <si>
+    <t>WA</t>
+  </si>
+  <si>
+    <t>West Virginia</t>
+  </si>
+  <si>
+    <t>WV</t>
+  </si>
+  <si>
+    <t>Wisconsin</t>
+  </si>
+  <si>
+    <t>WI</t>
+  </si>
+  <si>
+    <t>Wyoming</t>
+  </si>
+  <si>
+    <t>WY</t>
+  </si>
 </sst>
 </file>
 
@@ -368,7 +629,7 @@
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +695,25 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF403F41"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF403F41"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -464,7 +744,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -509,6 +789,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -865,143 +1156,510 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G51"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="70.81640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="70.86328125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="32">
+        <v>45051</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="B2" s="30" t="str">
+        <f>LOOKUP(B1,F2:G51,G2:G51)</f>
+        <v>PA</v>
+      </c>
+      <c r="F2" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="G2" s="31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F3" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" s="31" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B4" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F4" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B5" s="3">
         <v>2019</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F5" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5" s="31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B6" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F6" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B7" s="14" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F7" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="G7" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F8" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B9" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F9" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B10" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F10" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B11" s="3">
         <v>2022</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F11" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="G11" s="31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B12" s="3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F12" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F13" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="G13" s="31" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B14" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F14" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B15" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F15" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="G15" s="31" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B16" s="3">
         <v>2021</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F16" s="31" t="s">
+        <v>130</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B17" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F17" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B18" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F18" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F19" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="G19" s="31" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B20" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F20" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="G20" s="31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B21" s="3">
         <v>2022</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F21" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B22" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F22" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.75">
       <c r="B23" s="3" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F23" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="G23" s="31" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F24" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="G24" s="31" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F25" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="G25" s="31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A26" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F26" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="G26" s="31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F27" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="G27" s="31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A28" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F28" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A29" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="F29" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="G29" s="31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F30" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.75">
       <c r="A31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="F31" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F32" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="G32" s="31" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="59" x14ac:dyDescent="0.75">
       <c r="A33" s="16" t="s">
         <v>43</v>
       </c>
       <c r="B33">
         <v>0.88711067149387013</v>
       </c>
-      <c r="G33" s="9"/>
+      <c r="F33" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="G33" s="31" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F34" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" s="31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F35" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="G35" s="31" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F36" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="G36" s="31" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F37" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="G37" s="31" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F38" s="31" t="s">
+        <v>168</v>
+      </c>
+      <c r="G38" s="31" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F39" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="G39" s="31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F40" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="G40" s="31" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F41" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="G41" s="31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F42" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="G42" s="31" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F43" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="G43" s="31" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F44" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="G44" s="31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F45" s="31" t="s">
+        <v>180</v>
+      </c>
+      <c r="G45" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F46" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="G46" s="31" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F47" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="G47" s="31" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="F48" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="G48" s="31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="49" spans="6:7" x14ac:dyDescent="0.75">
+      <c r="F49" s="31" t="s">
+        <v>187</v>
+      </c>
+      <c r="G49" s="31" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="50" spans="6:7" x14ac:dyDescent="0.75">
+      <c r="F50" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="G50" s="31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="51" spans="6:7" x14ac:dyDescent="0.75">
+      <c r="F51" s="31" t="s">
+        <v>191</v>
+      </c>
+      <c r="G51" s="31" t="s">
+        <v>192</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1015,19 +1673,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB5E61F-7942-4515-8229-A2210CA98666}">
   <dimension ref="A1:AG57"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="45.36328125" customWidth="1"/>
+    <col min="1" max="1" width="45.40625" customWidth="1"/>
     <col min="2" max="2" width="15.7265625" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="3" max="3" width="19.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A2">
         <v>2020</v>
       </c>
@@ -1122,7 +1780,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A3" s="2">
         <f>'Baseline Calculations'!C104</f>
         <v>7491.2019000999289</v>
@@ -1248,31 +1906,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A8" s="18" t="s">
         <v>45</v>
       </c>
       <c r="B8" s="18"/>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A9" s="17" t="s">
         <v>46</v>
       </c>
@@ -1281,7 +1939,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A10" s="17" t="s">
         <v>48</v>
       </c>
@@ -1290,13 +1948,13 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A11" s="17" t="s">
         <v>50</v>
       </c>
       <c r="B11" s="17"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A12" s="17" t="s">
         <v>8</v>
       </c>
@@ -1334,7 +1992,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A13" s="17" t="s">
         <v>44</v>
       </c>
@@ -1345,31 +2003,31 @@
         <v>53</v>
       </c>
       <c r="D13" s="17">
-        <v>4750</v>
+        <v>2500</v>
       </c>
       <c r="E13" s="17">
-        <v>4750</v>
+        <v>2500</v>
       </c>
       <c r="F13" s="17">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="G13" s="17">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="H13" s="17">
-        <v>2400</v>
+        <v>2000</v>
       </c>
       <c r="I13" s="17">
-        <v>2400</v>
+        <v>2000</v>
       </c>
       <c r="J13" s="17">
-        <v>2400</v>
+        <v>2000</v>
       </c>
       <c r="K13" s="18" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A14" s="17" t="s">
         <v>55</v>
       </c>
@@ -1405,7 +2063,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.75">
       <c r="A15" s="17" t="s">
         <v>57</v>
       </c>
@@ -1416,33 +2074,33 @@
         <v>53</v>
       </c>
       <c r="D15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="E15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="F15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="H15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="I15" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="J15" s="17">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="16" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A16" s="17" t="s">
         <v>58</v>
       </c>
       <c r="B16" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="20" t="s">
         <v>53</v>
@@ -1474,7 +2132,7 @@
       <c r="L16" s="20"/>
       <c r="M16" s="22"/>
     </row>
-    <row r="17" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A17" s="17" t="s">
         <v>59</v>
       </c>
@@ -1488,10 +2146,10 @@
         <v>2500</v>
       </c>
       <c r="E17" s="17">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="F17" s="17">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="G17" s="17">
         <v>0</v>
@@ -1510,7 +2168,7 @@
       </c>
       <c r="R17" s="23"/>
     </row>
-    <row r="18" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A18" s="17" t="s">
         <v>61</v>
       </c>
@@ -1521,28 +2179,28 @@
         <v>53</v>
       </c>
       <c r="D18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="E18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="F18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="H18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="I18" s="17">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="J18" s="17">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="19" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A19" s="17" t="s">
         <v>62</v>
       </c>
@@ -1574,7 +2232,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="20" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A20" s="17" t="s">
         <v>63</v>
       </c>
@@ -1606,7 +2264,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="21" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A21" s="17" t="s">
         <v>64</v>
       </c>
@@ -1617,28 +2275,28 @@
         <v>53</v>
       </c>
       <c r="D21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="E21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="F21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="G21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="H21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="I21" s="17">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="J21" s="17">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="22" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A22" s="17" t="s">
         <v>65</v>
       </c>
@@ -1649,28 +2307,28 @@
         <v>53</v>
       </c>
       <c r="D22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="E22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="G22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="H22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="I22" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="J22" s="17">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="23" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A23" s="17" t="s">
         <v>66</v>
       </c>
@@ -1681,28 +2339,28 @@
         <v>53</v>
       </c>
       <c r="D23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="E23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="F23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="G23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="I23" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="J23" s="17">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A24" s="17" t="s">
         <v>67</v>
       </c>
@@ -1713,28 +2371,28 @@
         <v>53</v>
       </c>
       <c r="D24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="E24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="G24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="H24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="I24" s="17">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="J24" s="17">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="25" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A25" s="17" t="s">
         <v>68</v>
       </c>
@@ -1745,36 +2403,36 @@
         <v>53</v>
       </c>
       <c r="D25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="E25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="G25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="H25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="I25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="J25" s="17">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="K25" s="17" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A26" s="17" t="s">
         <v>71</v>
       </c>
       <c r="B26" s="17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17">
@@ -1800,7 +2458,7 @@
       </c>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A27" s="17" t="s">
         <v>70</v>
       </c>
@@ -1808,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -1820,20 +2478,24 @@
       <c r="I28" s="17"/>
       <c r="J28" s="18"/>
     </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A29" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A30" s="2"/>
     </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A31" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="B31" t="str">
+        <f>About!B2</f>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.75">
       <c r="C32">
         <v>2020</v>
       </c>
@@ -1928,132 +2590,132 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="33" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:33" x14ac:dyDescent="0.75">
       <c r="C33" s="2">
-        <f t="shared" ref="C33" si="1">SUMPRODUCT(D13:D26,$B$13:$B$26)/SUM($B$13:$B$26)</f>
+        <f>SUMIFS(D$13:D$26,$A$13:$A$26,$B$31)</f>
         <v>0</v>
       </c>
       <c r="D33" s="2">
-        <f t="shared" ref="D33" si="2">SUMPRODUCT(E13:E26,$B$13:$B$26)/SUM($B$13:$B$26)</f>
+        <f t="shared" ref="D33:I33" si="1">SUMIFS(E$13:E$26,$A$13:$A$26,$B$31)</f>
         <v>0</v>
       </c>
       <c r="E33" s="2">
-        <f t="shared" ref="E33" si="3">SUMPRODUCT(F13:F26,$B$13:$B$26)/SUM($B$13:$B$26)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F33" s="2">
-        <f t="shared" ref="F33" si="4">SUMPRODUCT(G13:G26,$B$13:$B$26)/SUM($B$13:$B$26)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G33" s="2">
-        <f t="shared" ref="G33:I33" si="5">SUMPRODUCT(H13:H26,$B$13:$B$26)/SUM($B$13:$B$26)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H33" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I33" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J33" s="2">
         <v>0</v>
       </c>
       <c r="K33" s="2">
-        <f t="shared" ref="K33:AG33" si="6">J33</f>
+        <f t="shared" ref="K33:AG33" si="2">J33</f>
         <v>0</v>
       </c>
       <c r="L33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="W33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AA33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AD33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF33" s="2">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AG33" s="2">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:33" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
         <v>103</v>
       </c>
@@ -2089,15 +2751,15 @@
       <c r="AF34" s="2"/>
       <c r="AG34" s="2"/>
     </row>
-    <row r="35" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A35" s="2"/>
     </row>
-    <row r="36" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A36" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:33" x14ac:dyDescent="0.75">
       <c r="C37">
         <v>2020</v>
       </c>
@@ -2192,7 +2854,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="38" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:33" x14ac:dyDescent="0.75">
       <c r="B38" s="2"/>
       <c r="C38" s="2">
         <f>(A3+C33)*About!$B$33</f>
@@ -2319,7 +2981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -2417,7 +3079,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="41" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -2515,12 +3177,12 @@
         <v>38175</v>
       </c>
     </row>
-    <row r="43" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A43" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:33" x14ac:dyDescent="0.75">
       <c r="C44">
         <v>2020</v>
       </c>
@@ -2615,7 +3277,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="45" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
@@ -2623,127 +3285,127 @@
         <v>0.18016388732564667</v>
       </c>
       <c r="D45" s="7">
-        <f t="shared" ref="D45:AG45" si="7">D38/C41</f>
+        <f t="shared" ref="D45:AG45" si="3">D38/C41</f>
         <v>0.1781803175643257</v>
       </c>
       <c r="E45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>9.6896533338125937E-2</v>
       </c>
       <c r="F45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>3.7939954068428282E-2</v>
       </c>
       <c r="G45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>2.2347138307484384E-2</v>
       </c>
       <c r="H45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>1.1189041060965108E-2</v>
       </c>
       <c r="I45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.977370947965275E-3</v>
       </c>
       <c r="J45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.972080493189055E-3</v>
       </c>
       <c r="K45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.9634193214199959E-3</v>
       </c>
       <c r="L45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.9516197902245803E-3</v>
       </c>
       <c r="M45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.9377580124603223E-3</v>
       </c>
       <c r="N45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.9224822279215408E-3</v>
       </c>
       <c r="O45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>6.4493098638198163E-3</v>
       </c>
       <c r="P45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>3.9230098371081726E-3</v>
       </c>
       <c r="Q45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>1.5268255803143347E-3</v>
       </c>
       <c r="R45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>3.042440593046421E-4</v>
       </c>
       <c r="S45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7969311125697645E-5</v>
       </c>
       <c r="T45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7924474237160522E-5</v>
       </c>
       <c r="U45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7904110875978027E-5</v>
       </c>
       <c r="V45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7889862854445594E-5</v>
       </c>
       <c r="W45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7900039480808213E-5</v>
       </c>
       <c r="X45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.790003948080824E-5</v>
       </c>
       <c r="Y45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7910218766753334E-5</v>
       </c>
       <c r="Z45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7934659910358932E-5</v>
       </c>
       <c r="AA45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7959116393594405E-5</v>
       </c>
       <c r="AB45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.7983588230905353E-5</v>
       </c>
       <c r="AC45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.8012158132910721E-5</v>
       </c>
       <c r="AD45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.8032578025626903E-5</v>
       </c>
       <c r="AE45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>7.8050965071110089E-5</v>
       </c>
       <c r="AF45" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>2.9274477036873986E-5</v>
       </c>
       <c r="AG45" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="2:12" x14ac:dyDescent="0.75">
       <c r="B57" s="10"/>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
@@ -2769,26 +3431,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC9C9DB8-910A-422D-8387-227BB59B1D40}">
   <dimension ref="A1:AI104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" customWidth="1"/>
+    <col min="1" max="1" width="51.86328125" customWidth="1"/>
     <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="36.453125" customWidth="1"/>
+    <col min="3" max="3" width="36.40625" customWidth="1"/>
     <col min="4" max="4" width="10.7265625" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" customWidth="1"/>
-    <col min="7" max="7" width="13.08984375" customWidth="1"/>
+    <col min="5" max="5" width="14.40625" customWidth="1"/>
+    <col min="6" max="6" width="11.86328125" customWidth="1"/>
+    <col min="7" max="7" width="13.1328125" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="10.7265625" customWidth="1"/>
-    <col min="10" max="10" width="11.81640625" customWidth="1"/>
+    <col min="10" max="10" width="11.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.75">
       <c r="D1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.75">
       <c r="B2">
         <v>2020</v>
       </c>
@@ -2883,7 +3545,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -3013,7 +3675,7 @@
       </c>
       <c r="AG3" s="11"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>81</v>
       </c>
@@ -3143,7 +3805,7 @@
       </c>
       <c r="AG4" s="11"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -3273,7 +3935,7 @@
       </c>
       <c r="AG5" s="11"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -3403,7 +4065,7 @@
       </c>
       <c r="AG6" s="11"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -3533,7 +4195,7 @@
       </c>
       <c r="AG7" s="11"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>82</v>
       </c>
@@ -3663,7 +4325,7 @@
       </c>
       <c r="AG8" s="11"/>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>83</v>
       </c>
@@ -3793,7 +4455,7 @@
       </c>
       <c r="AG9" s="11"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -3923,7 +4585,7 @@
       </c>
       <c r="AG10" s="11"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4053,7 +4715,7 @@
       </c>
       <c r="AG11" s="11"/>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -4183,7 +4845,7 @@
       </c>
       <c r="AG12" s="11"/>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -4313,7 +4975,7 @@
       </c>
       <c r="AG13" s="11"/>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>84</v>
       </c>
@@ -4443,7 +5105,7 @@
       </c>
       <c r="AG14" s="11"/>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -4575,7 +5237,7 @@
       <c r="AH15" s="11"/>
       <c r="AI15" s="11"/>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -4707,7 +5369,7 @@
       <c r="AH16" s="11"/>
       <c r="AI16" s="11"/>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>86</v>
       </c>
@@ -4839,7 +5501,7 @@
       <c r="AH17" s="11"/>
       <c r="AI17" s="11"/>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -4971,7 +5633,7 @@
       <c r="AH18" s="11"/>
       <c r="AI18" s="11"/>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -5103,7 +5765,7 @@
       <c r="AH19" s="11"/>
       <c r="AI19" s="11"/>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A20" t="s">
         <v>88</v>
       </c>
@@ -5235,7 +5897,7 @@
       <c r="AH20" s="11"/>
       <c r="AI20" s="11"/>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -5367,7 +6029,7 @@
       <c r="AH21" s="11"/>
       <c r="AI21" s="11"/>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -5499,7 +6161,7 @@
       <c r="AH22" s="11"/>
       <c r="AI22" s="11"/>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -5631,7 +6293,7 @@
       <c r="AH23" s="11"/>
       <c r="AI23" s="11"/>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -5763,7 +6425,7 @@
       <c r="AH24" s="11"/>
       <c r="AI24" s="11"/>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.75">
       <c r="B25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
@@ -5792,12 +6454,12 @@
       <c r="AG25" s="12"/>
       <c r="AH25" s="12"/>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A26" s="25" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -5895,7 +6557,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -5993,7 +6655,7 @@
         <v>11670000</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -6091,7 +6753,7 @@
         <v>1016090</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A31" s="1" t="s">
         <v>99</v>
       </c>
@@ -6189,7 +6851,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.75">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -6320,7 +6982,7 @@
       <c r="AG32" s="11"/>
       <c r="AH32" s="11"/>
     </row>
-    <row r="33" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A33" t="s">
         <v>81</v>
       </c>
@@ -6451,7 +7113,7 @@
       <c r="AG33" s="11"/>
       <c r="AH33" s="11"/>
     </row>
-    <row r="34" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -6582,7 +7244,7 @@
       <c r="AG34" s="11"/>
       <c r="AH34" s="11"/>
     </row>
-    <row r="35" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A35" t="s">
         <v>31</v>
       </c>
@@ -6713,7 +7375,7 @@
       <c r="AG35" s="11"/>
       <c r="AH35" s="11"/>
     </row>
-    <row r="36" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -6844,7 +7506,7 @@
       <c r="AG36" s="11"/>
       <c r="AH36" s="11"/>
     </row>
-    <row r="37" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A37" t="s">
         <v>82</v>
       </c>
@@ -6975,7 +7637,7 @@
       <c r="AG37" s="11"/>
       <c r="AH37" s="11"/>
     </row>
-    <row r="38" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A38" t="s">
         <v>83</v>
       </c>
@@ -7106,7 +7768,7 @@
       <c r="AG38" s="11"/>
       <c r="AH38" s="11"/>
     </row>
-    <row r="39" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A39" t="s">
         <v>24</v>
       </c>
@@ -7237,7 +7899,7 @@
       <c r="AG39" s="11"/>
       <c r="AH39" s="11"/>
     </row>
-    <row r="40" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
         <v>25</v>
       </c>
@@ -7368,7 +8030,7 @@
       <c r="AG40" s="11"/>
       <c r="AH40" s="11"/>
     </row>
-    <row r="41" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A41" t="s">
         <v>27</v>
       </c>
@@ -7499,7 +8161,7 @@
       <c r="AG41" s="11"/>
       <c r="AH41" s="11"/>
     </row>
-    <row r="42" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -7630,7 +8292,7 @@
       <c r="AG42" s="11"/>
       <c r="AH42" s="11"/>
     </row>
-    <row r="43" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -7761,7 +8423,7 @@
       <c r="AG43" s="11"/>
       <c r="AH43" s="11"/>
     </row>
-    <row r="44" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -7892,7 +8554,7 @@
       <c r="AG44" s="11"/>
       <c r="AH44" s="11"/>
     </row>
-    <row r="45" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A45" t="s">
         <v>85</v>
       </c>
@@ -8023,7 +8685,7 @@
       <c r="AG45" s="11"/>
       <c r="AH45" s="11"/>
     </row>
-    <row r="46" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -8154,7 +8816,7 @@
       <c r="AG46" s="11"/>
       <c r="AH46" s="11"/>
     </row>
-    <row r="47" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -8285,7 +8947,7 @@
       <c r="AG47" s="11"/>
       <c r="AH47" s="11"/>
     </row>
-    <row r="48" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A48" t="s">
         <v>87</v>
       </c>
@@ -8416,7 +9078,7 @@
       <c r="AG48" s="11"/>
       <c r="AH48" s="11"/>
     </row>
-    <row r="49" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A49" t="s">
         <v>88</v>
       </c>
@@ -8547,7 +9209,7 @@
       <c r="AG49" s="11"/>
       <c r="AH49" s="11"/>
     </row>
-    <row r="50" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A50" t="s">
         <v>32</v>
       </c>
@@ -8678,7 +9340,7 @@
       <c r="AG50" s="11"/>
       <c r="AH50" s="11"/>
     </row>
-    <row r="51" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A51" t="s">
         <v>73</v>
       </c>
@@ -8809,7 +9471,7 @@
       <c r="AG51" s="11"/>
       <c r="AH51" s="11"/>
     </row>
-    <row r="52" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A52" t="s">
         <v>74</v>
       </c>
@@ -8940,7 +9602,7 @@
       <c r="AG52" s="11"/>
       <c r="AH52" s="11"/>
     </row>
-    <row r="53" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A53" t="s">
         <v>72</v>
       </c>
@@ -9071,7 +9733,7 @@
       <c r="AG53" s="11"/>
       <c r="AH53" s="11"/>
     </row>
-    <row r="54" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:34" x14ac:dyDescent="0.75">
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
@@ -9106,7 +9768,7 @@
       <c r="AG54" s="11"/>
       <c r="AH54" s="11"/>
     </row>
-    <row r="55" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A55" s="1" t="s">
         <v>100</v>
       </c>
@@ -9204,7 +9866,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="56" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -9335,7 +9997,7 @@
       <c r="AG56" s="11"/>
       <c r="AH56" s="11"/>
     </row>
-    <row r="57" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A57" t="s">
         <v>81</v>
       </c>
@@ -9466,7 +10128,7 @@
       <c r="AG57" s="11"/>
       <c r="AH57" s="11"/>
     </row>
-    <row r="58" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A58" t="s">
         <v>11</v>
       </c>
@@ -9597,7 +10259,7 @@
       <c r="AG58" s="11"/>
       <c r="AH58" s="11"/>
     </row>
-    <row r="59" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A59" t="s">
         <v>31</v>
       </c>
@@ -9728,7 +10390,7 @@
       <c r="AG59" s="11"/>
       <c r="AH59" s="11"/>
     </row>
-    <row r="60" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A60" t="s">
         <v>26</v>
       </c>
@@ -9859,7 +10521,7 @@
       <c r="AG60" s="11"/>
       <c r="AH60" s="11"/>
     </row>
-    <row r="61" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A61" t="s">
         <v>82</v>
       </c>
@@ -9990,7 +10652,7 @@
       <c r="AG61" s="11"/>
       <c r="AH61" s="11"/>
     </row>
-    <row r="62" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A62" t="s">
         <v>83</v>
       </c>
@@ -10121,7 +10783,7 @@
       <c r="AG62" s="11"/>
       <c r="AH62" s="11"/>
     </row>
-    <row r="63" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -10252,7 +10914,7 @@
       <c r="AG63" s="11"/>
       <c r="AH63" s="11"/>
     </row>
-    <row r="64" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A64" t="s">
         <v>25</v>
       </c>
@@ -10383,7 +11045,7 @@
       <c r="AG64" s="11"/>
       <c r="AH64" s="11"/>
     </row>
-    <row r="65" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A65" t="s">
         <v>27</v>
       </c>
@@ -10514,7 +11176,7 @@
       <c r="AG65" s="11"/>
       <c r="AH65" s="11"/>
     </row>
-    <row r="66" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A66" t="s">
         <v>28</v>
       </c>
@@ -10645,7 +11307,7 @@
       <c r="AG66" s="11"/>
       <c r="AH66" s="11"/>
     </row>
-    <row r="67" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A67" t="s">
         <v>84</v>
       </c>
@@ -10776,7 +11438,7 @@
       <c r="AG67" s="11"/>
       <c r="AH67" s="11"/>
     </row>
-    <row r="68" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A68" t="s">
         <v>30</v>
       </c>
@@ -10907,7 +11569,7 @@
       <c r="AG68" s="11"/>
       <c r="AH68" s="11"/>
     </row>
-    <row r="69" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A69" t="s">
         <v>85</v>
       </c>
@@ -11038,7 +11700,7 @@
       <c r="AG69" s="11"/>
       <c r="AH69" s="11"/>
     </row>
-    <row r="70" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A70" t="s">
         <v>86</v>
       </c>
@@ -11169,7 +11831,7 @@
       <c r="AG70" s="11"/>
       <c r="AH70" s="11"/>
     </row>
-    <row r="71" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A71" t="s">
         <v>29</v>
       </c>
@@ -11300,7 +11962,7 @@
       <c r="AG71" s="11"/>
       <c r="AH71" s="11"/>
     </row>
-    <row r="72" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A72" t="s">
         <v>87</v>
       </c>
@@ -11431,7 +12093,7 @@
       <c r="AG72" s="11"/>
       <c r="AH72" s="11"/>
     </row>
-    <row r="73" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A73" t="s">
         <v>88</v>
       </c>
@@ -11562,7 +12224,7 @@
       <c r="AG73" s="11"/>
       <c r="AH73" s="11"/>
     </row>
-    <row r="74" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A74" t="s">
         <v>32</v>
       </c>
@@ -11693,7 +12355,7 @@
       <c r="AG74" s="11"/>
       <c r="AH74" s="11"/>
     </row>
-    <row r="75" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -11824,7 +12486,7 @@
       <c r="AG75" s="11"/>
       <c r="AH75" s="11"/>
     </row>
-    <row r="76" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A76" t="s">
         <v>74</v>
       </c>
@@ -11955,7 +12617,7 @@
       <c r="AG76" s="11"/>
       <c r="AH76" s="11"/>
     </row>
-    <row r="77" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A77" t="s">
         <v>72</v>
       </c>
@@ -12086,7 +12748,7 @@
       <c r="AG77" s="11"/>
       <c r="AH77" s="11"/>
     </row>
-    <row r="79" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A79" s="1" t="s">
         <v>102</v>
       </c>
@@ -12184,7 +12846,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="80" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:34" x14ac:dyDescent="0.75">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -12313,7 +12975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A81" t="s">
         <v>81</v>
       </c>
@@ -12442,7 +13104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -12571,7 +13233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A83" t="s">
         <v>31</v>
       </c>
@@ -12700,7 +13362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A84" t="s">
         <v>26</v>
       </c>
@@ -12829,7 +13491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A85" t="s">
         <v>82</v>
       </c>
@@ -12958,7 +13620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -13087,7 +13749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A87" t="s">
         <v>24</v>
       </c>
@@ -13216,7 +13878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A88" t="s">
         <v>25</v>
       </c>
@@ -13345,7 +14007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A89" t="s">
         <v>27</v>
       </c>
@@ -13474,7 +14136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A90" t="s">
         <v>28</v>
       </c>
@@ -13603,7 +14265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A91" t="s">
         <v>84</v>
       </c>
@@ -13732,7 +14394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A92" t="s">
         <v>30</v>
       </c>
@@ -13861,7 +14523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A93" t="s">
         <v>85</v>
       </c>
@@ -13990,7 +14652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A94" t="s">
         <v>86</v>
       </c>
@@ -14119,7 +14781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A95" t="s">
         <v>29</v>
       </c>
@@ -14248,7 +14910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A96" t="s">
         <v>87</v>
       </c>
@@ -14377,7 +15039,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="97" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A97" t="s">
         <v>88</v>
       </c>
@@ -14506,7 +15168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -14635,7 +15297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A99" t="s">
         <v>73</v>
       </c>
@@ -14764,7 +15426,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="100" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A100" t="s">
         <v>74</v>
       </c>
@@ -14893,7 +15555,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="101" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A101" t="s">
         <v>72</v>
       </c>
@@ -15022,7 +15684,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="103" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:33" x14ac:dyDescent="0.75">
       <c r="A103" t="s">
         <v>35</v>
       </c>
@@ -15120,7 +15782,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="104" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:33" x14ac:dyDescent="0.75">
       <c r="C104" s="13">
         <f>SUMPRODUCT(C80:C101,B56:B77)/SUM(B56:B77)</f>
         <v>7491.2019000999289</v>
@@ -15247,7 +15909,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AG3:AG14 B3:AF24 AG15:AI24">
+  <conditionalFormatting sqref="AG15:AI24 AG3:AG14 B3:AF24">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>B3&gt;600000</formula>
     </cfRule>
@@ -15263,23 +15925,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5680535D-1EA9-4EA0-BC79-B0A926B70A46}">
   <dimension ref="A1:Q81"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="21.1796875" customWidth="1"/>
+    <col min="1" max="1" width="21.1328125" customWidth="1"/>
     <col min="16" max="16" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A2" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A3" s="25" t="s">
         <v>90</v>
       </c>
@@ -15328,7 +15990,7 @@
       </c>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -15373,7 +16035,7 @@
         <v>0.506558531141579</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -15421,7 +16083,7 @@
         <v>3.9217017138996661E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -15469,7 +16131,7 @@
         <v>2.2475794205762668E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -15514,7 +16176,7 @@
         <v>8.3290977797280619E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -15559,7 +16221,7 @@
         <v>5.2458778329539747E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>82</v>
       </c>
@@ -15604,7 +16266,7 @@
         <v>3.6405767087696481E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -15646,7 +16308,7 @@
         <v>7.6907656512913439E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -15691,7 +16353,7 @@
         <v>3.654151526535612E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -15724,7 +16386,7 @@
         <v>3.159933451823603E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -15760,7 +16422,7 @@
         <v>2.6854462168877047E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -15799,7 +16461,7 @@
         <v>2.3072454800592241E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>84</v>
       </c>
@@ -15835,7 +16497,7 @@
         <v>4.0201980660620085E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -15877,7 +16539,7 @@
         <v>1.8832691949501677E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -15916,7 +16578,7 @@
         <v>2.6478786979539908E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
         <v>86</v>
       </c>
@@ -15955,7 +16617,7 @@
         <v>8.0028286131903035E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -16003,7 +16665,7 @@
         <v>3.5515511596998389E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A20" t="s">
         <v>87</v>
       </c>
@@ -16051,7 +16713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A21" t="s">
         <v>88</v>
       </c>
@@ -16078,7 +16740,7 @@
         <v>2.6281478581778807E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -16105,7 +16767,7 @@
         <v>4.1324270827085233E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -16123,7 +16785,7 @@
         <v>5.9350366046539526E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -16141,7 +16803,7 @@
         <v>1.0260036683577312E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -16159,7 +16821,7 @@
         <v>1.831021931223028E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -16203,12 +16865,12 @@
         <v>2693068</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A29" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A30" s="25" t="s">
         <v>90</v>
       </c>
@@ -16256,7 +16918,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -16302,7 +16964,7 @@
         <v>0.69848904985569582</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A32" t="s">
         <v>81</v>
       </c>
@@ -16351,7 +17013,7 @@
         <v>5.4041171323724657E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -16400,7 +17062,7 @@
         <v>3.0991672579584979E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -16446,7 +17108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -16492,7 +17154,7 @@
         <v>5.9247441483874057E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A36" t="s">
         <v>82</v>
       </c>
@@ -16538,7 +17200,7 @@
         <v>7.5852222023915757E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A37" t="s">
         <v>83</v>
       </c>
@@ -16581,7 +17243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A38" t="s">
         <v>24</v>
       </c>
@@ -16627,7 +17289,7 @@
         <v>2.1765343478885439E-6</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A39" t="s">
         <v>25</v>
       </c>
@@ -16661,7 +17323,7 @@
         <v>2.4107294437213513E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -16698,7 +17360,7 @@
         <v>2.3626280346330145E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -16738,7 +17400,7 @@
         <v>1.8972849910544438E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -16775,7 +17437,7 @@
         <v>2.146715827322471E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -16818,7 +17480,7 @@
         <v>2.0500777022762196E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A44" t="s">
         <v>85</v>
       </c>
@@ -16858,7 +17520,7 @@
         <v>3.6511363685830328E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -16898,7 +17560,7 @@
         <v>9.3373323524418542E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A46" t="s">
         <v>29</v>
       </c>
@@ -16947,7 +17609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A47" t="s">
         <v>87</v>
       </c>
@@ -16996,7 +17658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -17024,7 +17686,7 @@
         <v>2.3114794774576337E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A49" t="s">
         <v>32</v>
       </c>
@@ -17043,7 +17705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A50" t="s">
         <v>73</v>
       </c>
@@ -17062,7 +17724,7 @@
         <v>8.1837691480609253E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A51" t="s">
         <v>74</v>
       </c>
@@ -17081,7 +17743,7 @@
         <v>1.4147473261275537E-4</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A52" t="s">
         <v>72</v>
       </c>
@@ -17100,7 +17762,7 @@
         <v>2.5247798435507112E-4</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A54" t="s">
         <v>92</v>
       </c>
@@ -17153,12 +17815,12 @@
         <v>269433</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A56" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A57" s="25" t="s">
         <v>90</v>
       </c>
@@ -17206,7 +17868,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -17267,7 +17929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A59" t="s">
         <v>81</v>
       </c>
@@ -17328,7 +17990,7 @@
         <v>9.1911764705882352E-5</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A60" t="s">
         <v>11</v>
       </c>
@@ -17389,7 +18051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A61" t="s">
         <v>31</v>
       </c>
@@ -17450,7 +18112,7 @@
         <v>0.30311925551470587</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A62" t="s">
         <v>26</v>
       </c>
@@ -17511,7 +18173,7 @@
         <v>3.4541590073529409E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A63" t="s">
         <v>82</v>
       </c>
@@ -17572,7 +18234,7 @@
         <v>0.11247127757352941</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -17633,7 +18295,7 @@
         <v>0.27988855698529413</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -17694,7 +18356,7 @@
         <v>1.3292738970588235E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A66" t="s">
         <v>25</v>
       </c>
@@ -17755,7 +18417,7 @@
         <v>5.1372931985294121E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A67" t="s">
         <v>27</v>
       </c>
@@ -17816,7 +18478,7 @@
         <v>3.5374540441176473E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A68" t="s">
         <v>28</v>
       </c>
@@ -17877,7 +18539,7 @@
         <v>3.3892463235294115E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A69" t="s">
         <v>84</v>
       </c>
@@ -17938,7 +18600,7 @@
         <v>8.9648437499999997E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A70" t="s">
         <v>30</v>
       </c>
@@ -17999,7 +18661,7 @@
         <v>1.443014705882353E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A71" t="s">
         <v>85</v>
       </c>
@@ -18060,7 +18722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A72" t="s">
         <v>86</v>
       </c>
@@ -18121,7 +18783,7 @@
         <v>4.4806985294117645E-4</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A73" t="s">
         <v>29</v>
       </c>
@@ -18182,7 +18844,7 @@
         <v>1.2925091911764705E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A74" t="s">
         <v>87</v>
       </c>
@@ -18243,7 +18905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A75" t="s">
         <v>88</v>
       </c>
@@ -18304,7 +18966,7 @@
         <v>3.463924632352941E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A76" t="s">
         <v>32</v>
       </c>
@@ -18365,7 +19027,7 @@
         <v>1.50390625E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A77" t="s">
         <v>73</v>
       </c>
@@ -18426,7 +19088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A78" t="s">
         <v>74</v>
       </c>
@@ -18487,7 +19149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A79" t="s">
         <v>72</v>
       </c>
@@ -18548,7 +19210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A81" t="s">
         <v>92</v>
       </c>
@@ -18612,12 +19274,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="15.36328125" customWidth="1"/>
+    <col min="1" max="1" width="15.40625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A1" s="15" t="s">
         <v>41</v>
       </c>
@@ -18715,7 +19377,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -18844,7 +19506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -18942,7 +19604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -19040,7 +19702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -19138,7 +19800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -19236,7 +19898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -19345,12 +20007,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="16.81640625" customWidth="1"/>
+    <col min="1" max="1" width="16.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A1" s="15" t="s">
         <v>41</v>
       </c>
@@ -19448,7 +20110,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -19546,7 +20208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -19644,7 +20306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -19742,7 +20404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -19840,7 +20502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -19938,7 +20600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>21</v>
       </c>

</xml_diff>